<commit_message>
fix file import dot 2
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_matrix_cai_tao_bo_sung.xlsx
+++ b/docs/SLMS2026_import_matrix_cai_tao_bo_sung.xlsx
@@ -853,7 +853,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -866,7 +866,8 @@
     <col min="9" max="9" width="21.83203125" customWidth="1"/>
     <col min="10" max="10" width="25.83203125" customWidth="1"/>
     <col min="11" max="11" width="21.83203125" customWidth="1"/>
-    <col min="12" max="12" width="19.83203125" customWidth="1"/>
+    <col min="12" max="12" width="31.83203125" customWidth="1"/>
+    <col min="13" max="13" width="19.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -904,6 +905,9 @@
         <v>Ngày hết bảo hành</v>
       </c>
       <c r="L1" t="str">
+        <v>Giá phạt hết bảo hành (VNĐ)</v>
+      </c>
+      <c r="M1" t="str">
         <v>Ghi chú lắp đặt</v>
       </c>
     </row>
@@ -941,7 +945,10 @@
       <c r="K2" t="str">
         <v>2027-12-31</v>
       </c>
-      <c r="L2" t="str">
+      <c r="L2">
+        <v>270000</v>
+      </c>
+      <c r="M2" t="str">
         <v>SUPP#2 chỉ TB THEM_MOI</v>
       </c>
     </row>
@@ -979,7 +986,10 @@
       <c r="K3" t="str">
         <v>2030-01-31</v>
       </c>
-      <c r="L3" t="str">
+      <c r="L3">
+        <v>4650000</v>
+      </c>
+      <c r="M3" t="str">
         <v>SUPP#3 THAY_THE</v>
       </c>
     </row>
@@ -1017,13 +1027,16 @@
       <c r="K4" t="str">
         <v>2029-02-28</v>
       </c>
-      <c r="L4" t="str">
+      <c r="L4">
+        <v>2940000</v>
+      </c>
+      <c r="M4" t="str">
         <v>SUPP#4 THAY_THE phòng 102</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new file import excel
</commit_message>
<xml_diff>
--- a/docs/SLMS2026_import_matrix_cai_tao_bo_sung.xlsx
+++ b/docs/SLMS2026_import_matrix_cai_tao_bo_sung.xlsx
@@ -418,7 +418,7 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Dùng SAU KHI nhà #4, #6, #10 đã ACTIVE (host xác nhận + gán OM).</v>
+        <v>Dùng SAU KHI nhà #1, #2, #15, #41 đã ACTIVE (host xác nhận + gán OM).</v>
       </c>
     </row>
     <row r="4">
@@ -480,7 +480,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>HD-MTX-06-RENO-WH-HO-EQUIP</v>
+        <v>HD-MTX-01-RENO-WH-FULL</v>
       </c>
       <c r="C2" t="str">
         <v>Có</v>
@@ -500,7 +500,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>HD-MTX-04-RENO-WH-EQUIP</v>
+        <v>HD-MTX-15-RENO-WH-BASIC</v>
       </c>
       <c r="C3" t="str">
         <v>Không</v>
@@ -512,7 +512,7 @@
         <v>THEM_MOI</v>
       </c>
       <c r="F3" t="str">
-        <v>SUPP chỉ thêm TB mới</v>
+        <v>SUPP chỉ thêm quạt mới</v>
       </c>
     </row>
     <row r="4">
@@ -520,7 +520,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>HD-MTX-06-RENO-WH-HO-EQUIP</v>
+        <v>HD-MTX-02-RENO-WH-FULL</v>
       </c>
       <c r="C4" t="str">
         <v>Không</v>
@@ -532,7 +532,7 @@
         <v>THAY_THE</v>
       </c>
       <c r="F4" t="str">
-        <v>SUPP thay TB đã mua đợt 2</v>
+        <v>SUPP thay ĐH đã mua đợt 2</v>
       </c>
     </row>
     <row r="5">
@@ -540,7 +540,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>HD-MTX-10-RENO-RM-HO-EQUIP</v>
+        <v>HD-MTX-41-RENO-RM-FULL</v>
       </c>
       <c r="C5" t="str">
         <v>Có</v>
@@ -552,7 +552,7 @@
         <v>THAY_THE</v>
       </c>
       <c r="F5" t="str">
-        <v>SUPP cải tạo + thay TB phòng 102</v>
+        <v>SUPP cải tạo + thay ĐH phòng 102</v>
       </c>
     </row>
     <row r="6">
@@ -574,7 +574,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -708,76 +708,132 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Giường</v>
+        <v>Bàn ăn</v>
       </c>
       <c r="B14" t="str">
-        <v>Giường ngủ các loại</v>
+        <v>Bàn ăn và ghế</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Nóng lạnh</v>
+        <v>Giường</v>
       </c>
       <c r="B15" t="str">
-        <v>Máy nước nóng</v>
+        <v>Giường ngủ các loại</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Quạt</v>
+        <v>Tủ quần áo</v>
       </c>
       <c r="B16" t="str">
-        <v>Quạt điện / quạt trần</v>
+        <v>Tủ đựng quần áo</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
+        <v>Bếp từ</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Bếp từ / bếp gas</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Mã khu vực</v>
+        <v>Nóng lạnh</v>
       </c>
       <c r="B18" t="str">
-        <v>Mô tả</v>
+        <v>Máy nước nóng</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>LIVING_ROOM</v>
+        <v>Quạt</v>
       </c>
       <c r="B19" t="str">
-        <v>Phòng khách</v>
+        <v>Quạt điện / quạt trần</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>KITCHEN</v>
+        <v>Khác</v>
       </c>
       <c r="B20" t="str">
-        <v>Nhà bếp</v>
+        <v>Thiết bị khác</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>BATHROOM</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Phòng tắm / WC</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>Mã khu vực</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Mô tả</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>LIVING_ROOM</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Phòng khách</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>BEDROOM</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Phòng ngủ</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>KITCHEN</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Nhà bếp</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>BATHROOM</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Phòng tắm / WC</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v>BALCONY</v>
       </c>
-      <c r="B22" t="str">
+      <c r="B27" t="str">
         <v>Ban công</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>GARAGE</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Gara / sân</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>OTHER</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Khu vực khác</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -812,7 +868,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>HD-MTX-06-RENO-WH-HO-EQUIP</v>
+        <v>HD-MTX-01-RENO-WH-FULL</v>
       </c>
       <c r="B2" t="str">
         <v>OTHER</v>
@@ -824,12 +880,12 @@
         <v>3000000</v>
       </c>
       <c r="E2" t="str">
-        <v>SUPP#1 chỉ cải tạo</v>
+        <v>SUPP#1 chỉ cải tạo — sau khi nhà ACTIVE</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>HD-MTX-10-RENO-RM-HO-EQUIP</v>
+        <v>HD-MTX-41-RENO-RM-FULL</v>
       </c>
       <c r="B3" t="str">
         <v>PAINTING</v>
@@ -913,7 +969,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>HD-MTX-04-RENO-WH-EQUIP</v>
+        <v>HD-MTX-02-RENO-WH-FULL</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -922,39 +978,39 @@
         <v>LIVING_ROOM</v>
       </c>
       <c r="D2" t="str">
-        <v>Quạt</v>
+        <v>Điều hòa</v>
       </c>
       <c r="E2" t="str">
         <v>NEW</v>
       </c>
       <c r="F2" t="str">
-        <v>THEM_MOI</v>
+        <v>THAY_THE</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2">
-        <v>900000</v>
+        <v>15500000</v>
       </c>
       <c r="I2">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="J2" t="str">
-        <v>2027-01-01</v>
+        <v>2027-02-01</v>
       </c>
       <c r="K2" t="str">
-        <v>2027-12-31</v>
+        <v>2030-01-31</v>
       </c>
       <c r="L2">
-        <v>270000</v>
+        <v>4650000</v>
       </c>
       <c r="M2" t="str">
-        <v>SUPP#2 chỉ TB THEM_MOI</v>
+        <v>SUPP#3 THAY_THE ĐH phòng khách</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>HD-MTX-06-RENO-WH-HO-EQUIP</v>
+        <v>HD-MTX-15-RENO-WH-BASIC</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -963,39 +1019,39 @@
         <v>LIVING_ROOM</v>
       </c>
       <c r="D3" t="str">
-        <v>Điều hòa</v>
+        <v>Quạt</v>
       </c>
       <c r="E3" t="str">
         <v>NEW</v>
       </c>
       <c r="F3" t="str">
-        <v>THAY_THE</v>
+        <v>THEM_MOI</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3">
-        <v>15500000</v>
+        <v>900000</v>
       </c>
       <c r="I3">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="J3" t="str">
-        <v>2027-02-01</v>
+        <v>2027-01-01</v>
       </c>
       <c r="K3" t="str">
-        <v>2030-01-31</v>
+        <v>2027-12-31</v>
       </c>
       <c r="L3">
-        <v>4650000</v>
+        <v>270000</v>
       </c>
       <c r="M3" t="str">
-        <v>SUPP#3 THAY_THE</v>
+        <v>SUPP#2 chỉ TB THEM_MOI</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>HD-MTX-10-RENO-RM-HO-EQUIP</v>
+        <v>HD-MTX-41-RENO-RM-FULL</v>
       </c>
       <c r="B4" t="str">
         <v>102</v>

</xml_diff>